<commit_message>
2d, full, threshold, run probability on test/full set
</commit_message>
<xml_diff>
--- a/Result/Experiments_AML.xlsx
+++ b/Result/Experiments_AML.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://smu-my.sharepoint.com/personal/kh_nguyen_2025_mitb_smu_edu_sg/Documents/Data_Science/SMU/Study/Term 2/CS610 Applied ML/Project/Result/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="205" documentId="8_{95C4CE0D-2520-4E0B-A98D-599385999CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A82DB10-4398-4EA7-9065-9AEAD0355701}"/>
+  <xr:revisionPtr revIDLastSave="232" documentId="8_{95C4CE0D-2520-4E0B-A98D-599385999CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD178AB6-D33A-4D00-A5B5-3C3A41ABE878}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{3AEB3263-0B0E-46D1-87D0-7CDB5ACB019C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{3AEB3263-0B0E-46D1-87D0-7CDB5ACB019C}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="OptunaOPTUNA SEARCH COMPLETE" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Experiments (official)'!$A$1:$N$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Experiments (official)'!$A$1:$O$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="37">
   <si>
     <t>D_MODEL</t>
   </si>
@@ -257,6 +257,12 @@
   </si>
   <si>
     <t>rul_10d</t>
+  </si>
+  <si>
+    <t>N_HEAD</t>
+  </si>
+  <si>
+    <t>OPTUNA, lock D_model = 256, DIM_FEEDFORWARD = 1024=&gt; full_lr: 2.50e-05   (subset best 1.00e-04 / 4)</t>
   </si>
 </sst>
 </file>
@@ -378,13 +384,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>541020</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>76162</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>158548</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>33801</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -422,13 +428,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>1</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>281941</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:row>30</xdr:row>
       <xdr:rowOff>167179</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -466,13 +472,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>7621</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>173382</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>403860</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>49</xdr:row>
       <xdr:rowOff>155531</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -510,13 +516,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>1</xdr:colOff>
-      <xdr:row>63</xdr:row>
+      <xdr:row>64</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>594361</xdr:colOff>
-      <xdr:row>71</xdr:row>
+      <xdr:row>72</xdr:row>
       <xdr:rowOff>117857</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -554,13 +560,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>49</xdr:row>
+      <xdr:row>50</xdr:row>
       <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>60</xdr:row>
+      <xdr:row>61</xdr:row>
       <xdr:rowOff>63221</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -598,13 +604,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>45721</xdr:colOff>
-      <xdr:row>73</xdr:row>
+      <xdr:row>74</xdr:row>
       <xdr:rowOff>45084</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>495301</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>85</xdr:row>
       <xdr:rowOff>127269</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -642,13 +648,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>45721</xdr:colOff>
-      <xdr:row>85</xdr:row>
+      <xdr:row>86</xdr:row>
       <xdr:rowOff>130585</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>480061</xdr:colOff>
-      <xdr:row>98</xdr:row>
+      <xdr:row>99</xdr:row>
       <xdr:rowOff>176749</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1073,7 +1079,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E2361BB-17A0-4C3F-9B6A-2513337F59A8}">
-  <dimension ref="A1:N87"/>
+  <dimension ref="A1:P88"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="12.5546875" customWidth="1"/>
@@ -1085,7 +1091,7 @@
     <col min="11" max="11" width="12.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1105,31 +1111,34 @@
         <v>20</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1148,32 +1157,35 @@
       <c r="F2" s="6">
         <v>5</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="6">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2">
         <v>4</v>
       </c>
-      <c r="H2" s="2">
+      <c r="I2" s="2">
         <v>0.1</v>
       </c>
-      <c r="I2" s="2">
+      <c r="J2" s="2">
         <v>512</v>
       </c>
-      <c r="J2" s="2">
+      <c r="K2" s="2">
         <v>0.52780000000000005</v>
       </c>
-      <c r="K2" s="2">
+      <c r="L2" s="2">
         <v>0.34549999999999997</v>
       </c>
-      <c r="L2" s="2">
+      <c r="M2" s="2">
         <v>1</v>
       </c>
-      <c r="M2" s="2">
+      <c r="N2" s="2">
         <v>0.54449999999999998</v>
       </c>
-      <c r="N2" s="2">
+      <c r="O2" s="2">
         <v>0.51190000000000002</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1192,32 +1204,35 @@
       <c r="F3" s="6">
         <v>10</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="6">
+        <v>8</v>
+      </c>
+      <c r="H3" s="2">
         <v>4</v>
       </c>
-      <c r="H3" s="2">
+      <c r="I3" s="2">
         <v>0.1</v>
       </c>
-      <c r="I3" s="2">
+      <c r="J3" s="2">
         <v>512</v>
       </c>
-      <c r="J3" s="2">
+      <c r="K3" s="2">
         <v>0.59719999999999995</v>
       </c>
-      <c r="K3" s="2">
+      <c r="L3" s="2">
         <v>0.59340000000000004</v>
       </c>
-      <c r="L3" s="2">
+      <c r="M3" s="2">
         <v>0.65790000000000004</v>
       </c>
-      <c r="M3" s="2">
+      <c r="N3" s="2">
         <v>0.60529999999999995</v>
       </c>
-      <c r="N3" s="2">
+      <c r="O3" s="2">
         <v>0.57250000000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1236,32 +1251,35 @@
       <c r="F4" s="6">
         <v>15</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="6">
+        <v>8</v>
+      </c>
+      <c r="H4" s="2">
         <v>4</v>
       </c>
-      <c r="H4" s="2">
+      <c r="I4" s="2">
         <v>0.15</v>
       </c>
-      <c r="I4" s="2">
+      <c r="J4" s="2">
         <v>512</v>
       </c>
-      <c r="J4" s="2">
+      <c r="K4" s="2">
         <v>0.66669999999999996</v>
       </c>
-      <c r="K4" s="2">
+      <c r="L4" s="2">
         <v>0.66010000000000002</v>
       </c>
-      <c r="L4" s="2">
+      <c r="M4" s="2">
         <v>0.76319999999999999</v>
       </c>
-      <c r="M4" s="2">
+      <c r="N4" s="2">
         <v>0.72060000000000002</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>0.66590000000000005</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1280,81 +1298,82 @@
       <c r="F5" s="6">
         <v>10</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="6">
+        <v>8</v>
+      </c>
+      <c r="H5" s="2">
         <v>4</v>
       </c>
-      <c r="H5" s="2">
+      <c r="I5" s="2">
         <v>0.1</v>
       </c>
-      <c r="I5" s="2">
+      <c r="J5" s="2">
         <v>1024</v>
       </c>
-      <c r="J5" s="2">
+      <c r="K5" s="2">
         <v>0.69440000000000002</v>
       </c>
-      <c r="K5" s="2">
+      <c r="L5" s="2">
         <v>0.69350000000000001</v>
       </c>
-      <c r="L5" s="2">
+      <c r="M5" s="2">
         <v>0.60529999999999995</v>
       </c>
-      <c r="M5" s="2">
+      <c r="N5" s="2">
         <v>0.73680000000000001</v>
       </c>
-      <c r="N5">
+      <c r="O5">
         <v>0.73119999999999996</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C6" s="2">
-        <v>9212</v>
+        <v>2000</v>
       </c>
       <c r="D6" s="2">
         <v>256</v>
       </c>
       <c r="E6" s="7">
-        <v>3.0000000000000001E-5</v>
+        <v>1E-4</v>
       </c>
       <c r="F6" s="6">
         <v>10</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="6">
+        <v>8</v>
+      </c>
+      <c r="H6" s="2">
         <v>4</v>
       </c>
-      <c r="H6" s="2">
+      <c r="I6" s="2">
         <v>0.1</v>
       </c>
-      <c r="I6" s="2">
+      <c r="J6" s="2">
         <v>1024</v>
       </c>
-      <c r="J6" s="2">
-        <v>0.69699999999999995</v>
-      </c>
-      <c r="K6" s="2">
-        <v>0.67889999999999995</v>
-      </c>
-      <c r="L6" s="2">
-        <v>0.56889999999999996</v>
-      </c>
-      <c r="M6" s="2">
-        <v>0.75790000000000002</v>
-      </c>
-      <c r="N6" s="9">
-        <v>0.81610000000000005</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6">
+        <v>0.64329999999999998</v>
+      </c>
+      <c r="P6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C7" s="2">
         <v>9212</v>
@@ -1368,37 +1387,40 @@
       <c r="F7" s="6">
         <v>10</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="6">
+        <v>8</v>
+      </c>
+      <c r="H7" s="2">
         <v>4</v>
       </c>
-      <c r="H7" s="2">
+      <c r="I7" s="2">
         <v>0.1</v>
       </c>
-      <c r="I7" s="2">
+      <c r="J7" s="2">
         <v>1024</v>
       </c>
-      <c r="J7" s="2">
-        <v>0.74</v>
-      </c>
       <c r="K7" s="2">
-        <v>0.73939999999999995</v>
+        <v>0.69699999999999995</v>
       </c>
       <c r="L7" s="2">
-        <v>0.76670000000000005</v>
+        <v>0.67889999999999995</v>
       </c>
       <c r="M7" s="2">
-        <v>0.81</v>
-      </c>
-      <c r="N7" s="9">
-        <v>0.80779999999999996</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+        <v>0.56889999999999996</v>
+      </c>
+      <c r="N7" s="2">
+        <v>0.75790000000000002</v>
+      </c>
+      <c r="O7" s="9">
+        <v>0.81610000000000005</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C8" s="2">
         <v>9212</v>
@@ -1412,77 +1434,160 @@
       <c r="F8" s="6">
         <v>10</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="6">
+        <v>8</v>
+      </c>
+      <c r="H8" s="2">
         <v>4</v>
       </c>
-      <c r="H8" s="2">
+      <c r="I8" s="2">
         <v>0.1</v>
       </c>
-      <c r="I8" s="2">
+      <c r="J8" s="2">
         <v>1024</v>
       </c>
-      <c r="J8" s="2">
+      <c r="K8" s="2">
+        <v>0.74</v>
+      </c>
+      <c r="L8" s="2">
+        <v>0.73939999999999995</v>
+      </c>
+      <c r="M8" s="2">
+        <v>0.76670000000000005</v>
+      </c>
+      <c r="N8" s="2">
+        <v>0.81</v>
+      </c>
+      <c r="O8" s="9">
+        <v>0.80779999999999996</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="2">
+        <v>9212</v>
+      </c>
+      <c r="D9" s="2">
+        <v>256</v>
+      </c>
+      <c r="E9" s="7">
+        <v>3.0000000000000001E-5</v>
+      </c>
+      <c r="F9" s="6">
+        <v>10</v>
+      </c>
+      <c r="G9" s="6">
+        <v>8</v>
+      </c>
+      <c r="H9" s="2">
+        <v>4</v>
+      </c>
+      <c r="I9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J9" s="2">
+        <v>1024</v>
+      </c>
+      <c r="K9" s="2">
         <v>0.74719999999999998</v>
       </c>
-      <c r="K8" s="2">
+      <c r="L9" s="2">
         <v>0.74570000000000003</v>
       </c>
-      <c r="L8" s="2">
+      <c r="M9" s="2">
         <v>0.77459999999999996</v>
       </c>
-      <c r="M8" s="2">
+      <c r="N9" s="2">
         <v>0.81940000000000002</v>
       </c>
-      <c r="N8" s="9">
+      <c r="O9" s="9">
         <v>0.81110000000000004</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="2">
+        <v>9212</v>
+      </c>
+      <c r="D10" s="2">
+        <v>256</v>
+      </c>
+      <c r="E10" s="7">
+        <v>3.0000000000000001E-5</v>
+      </c>
+      <c r="F10" s="6">
+        <v>10</v>
+      </c>
+      <c r="G10" s="6">
+        <v>8</v>
+      </c>
+      <c r="H10" s="2">
+        <v>4</v>
+      </c>
+      <c r="I10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J10" s="2">
+        <v>1024</v>
+      </c>
+      <c r="K10" s="2">
+        <v>0.69869999999999999</v>
+      </c>
+      <c r="L10" s="2">
+        <v>0.68010000000000004</v>
+      </c>
+      <c r="M10" s="2">
+        <v>0.56640000000000001</v>
+      </c>
+      <c r="N10" s="2">
+        <v>0.75860000000000005</v>
+      </c>
+      <c r="O10" s="9">
+        <v>0.81630000000000003</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A74" t="s">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A87" t="s">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>